<commit_message>
fix: WEEK() formula on yearly calendar
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/yearly_calendar.xlsx
+++ b/xlsx/tests/templates/yearly_calendar.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/v0.8.02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02E46D9-EFAE-9744-B9A0-DAB4517D2AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88D010F-C510-4B4C-B6B5-F84C4CC698E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3900" yWindow="-19400" windowWidth="33960" windowHeight="17260" xr2:uid="{6F0581DF-A6A1-8847-8CD1-D7A1DAEC65B8}"/>
   </bookViews>
@@ -831,119 +831,95 @@
     </row>
     <row r="5" spans="1:33" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$5),"dddd"),1)</f>
+      <c r="B5" s="2" t="str" cm="1">
+        <f t="array" ref="B5:H5">week()</f>
         <v>M</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f t="shared" ref="C5:H5" si="0">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="D5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>W</v>
       </c>
       <c r="E5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>T</v>
       </c>
       <c r="F5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>F</v>
       </c>
       <c r="G5" s="12" t="str">
-        <f t="shared" si="0"/>
         <v>S</v>
       </c>
       <c r="H5" s="12" t="str">
-        <f t="shared" si="0"/>
         <v>S</v>
       </c>
       <c r="I5" s="11"/>
-      <c r="J5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$5),"dddd"),1)</f>
+      <c r="J5" s="2" t="str" cm="1">
+        <f t="array" ref="J5:P5">week()</f>
         <v>M</v>
       </c>
       <c r="K5" s="2" t="str">
-        <f t="shared" ref="K5:P5" si="1">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="L5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>W</v>
       </c>
       <c r="M5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>T</v>
       </c>
       <c r="N5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>F</v>
       </c>
       <c r="O5" s="12" t="str">
-        <f t="shared" si="1"/>
         <v>S</v>
       </c>
       <c r="P5" s="12" t="str">
-        <f t="shared" si="1"/>
         <v>S</v>
       </c>
       <c r="Q5" s="11"/>
-      <c r="R5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$5),"dddd"),1)</f>
+      <c r="R5" s="2" t="str" cm="1">
+        <f t="array" ref="R5:X5">week()</f>
         <v>M</v>
       </c>
       <c r="S5" s="2" t="str">
-        <f t="shared" ref="S5:X5" si="2">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="T5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>W</v>
       </c>
       <c r="U5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>T</v>
       </c>
       <c r="V5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>F</v>
       </c>
       <c r="W5" s="12" t="str">
-        <f t="shared" si="2"/>
         <v>S</v>
       </c>
       <c r="X5" s="12" t="str">
-        <f t="shared" si="2"/>
         <v>S</v>
       </c>
       <c r="Y5" s="11"/>
-      <c r="Z5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$5),"dddd"),1)</f>
+      <c r="Z5" s="2" t="str" cm="1">
+        <f t="array" ref="Z5:AF5">week()</f>
         <v>M</v>
       </c>
       <c r="AA5" s="2" t="str">
-        <f t="shared" ref="AA5:AF5" si="3">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="AB5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>W</v>
       </c>
       <c r="AC5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>T</v>
       </c>
       <c r="AD5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>F</v>
       </c>
       <c r="AE5" s="12" t="str">
-        <f t="shared" si="3"/>
         <v>S</v>
       </c>
       <c r="AF5" s="12" t="str">
-        <f t="shared" si="3"/>
         <v>S</v>
       </c>
       <c r="AG5" s="9"/>
@@ -1746,119 +1722,95 @@
     </row>
     <row r="14" spans="1:33" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$14),"dddd"),1)</f>
+      <c r="B14" s="2" t="str" cm="1">
+        <f t="array" ref="B14:H14">week()</f>
         <v>M</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f t="shared" ref="C14:H14" si="4">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$14),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="D14" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>W</v>
       </c>
       <c r="E14" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>T</v>
       </c>
       <c r="F14" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>F</v>
       </c>
       <c r="G14" s="12" t="str">
-        <f t="shared" si="4"/>
         <v>S</v>
       </c>
       <c r="H14" s="12" t="str">
-        <f t="shared" si="4"/>
         <v>S</v>
       </c>
       <c r="I14" s="11"/>
-      <c r="J14" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$14),"dddd"),1)</f>
+      <c r="J14" s="2" t="str" cm="1">
+        <f t="array" ref="J14:P14">week()</f>
         <v>M</v>
       </c>
       <c r="K14" s="2" t="str">
-        <f t="shared" ref="K14:P14" si="5">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$14),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="L14" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>W</v>
       </c>
       <c r="M14" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>T</v>
       </c>
       <c r="N14" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>F</v>
       </c>
       <c r="O14" s="12" t="str">
-        <f t="shared" si="5"/>
         <v>S</v>
       </c>
       <c r="P14" s="12" t="str">
-        <f t="shared" si="5"/>
         <v>S</v>
       </c>
       <c r="Q14" s="11"/>
-      <c r="R14" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$14),"dddd"),1)</f>
+      <c r="R14" s="2" t="str" cm="1">
+        <f t="array" ref="R14:X14">week()</f>
         <v>M</v>
       </c>
       <c r="S14" s="2" t="str">
-        <f t="shared" ref="S14:X14" si="6">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$14),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="T14" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>W</v>
       </c>
       <c r="U14" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>T</v>
       </c>
       <c r="V14" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>F</v>
       </c>
       <c r="W14" s="12" t="str">
-        <f t="shared" si="6"/>
         <v>S</v>
       </c>
       <c r="X14" s="12" t="str">
-        <f t="shared" si="6"/>
         <v>S</v>
       </c>
       <c r="Y14" s="11"/>
-      <c r="Z14" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$14),"dddd"),1)</f>
+      <c r="Z14" s="2" t="str" cm="1">
+        <f t="array" ref="Z14:AF14">week()</f>
         <v>M</v>
       </c>
       <c r="AA14" s="2" t="str">
-        <f t="shared" ref="AA14:AF14" si="7">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$14),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="AB14" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>W</v>
       </c>
       <c r="AC14" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>T</v>
       </c>
       <c r="AD14" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>F</v>
       </c>
       <c r="AE14" s="12" t="str">
-        <f t="shared" si="7"/>
         <v>S</v>
       </c>
       <c r="AF14" s="12" t="str">
-        <f t="shared" si="7"/>
         <v>S</v>
       </c>
       <c r="AG14" s="9"/>
@@ -2660,119 +2612,95 @@
     </row>
     <row r="23" spans="1:33" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$23),"dddd"),1)</f>
+      <c r="B23" s="2" t="str" cm="1">
+        <f t="array" ref="B23:H23">week()</f>
         <v>M</v>
       </c>
       <c r="C23" s="2" t="str">
-        <f t="shared" ref="C23:H23" si="8">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$23),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="D23" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>W</v>
       </c>
       <c r="E23" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>T</v>
       </c>
       <c r="F23" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>F</v>
       </c>
       <c r="G23" s="12" t="str">
-        <f t="shared" si="8"/>
         <v>S</v>
       </c>
       <c r="H23" s="12" t="str">
-        <f t="shared" si="8"/>
         <v>S</v>
       </c>
       <c r="I23" s="11"/>
-      <c r="J23" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$23),"dddd"),1)</f>
+      <c r="J23" s="2" t="str" cm="1">
+        <f t="array" ref="J23:P23">week()</f>
         <v>M</v>
       </c>
       <c r="K23" s="2" t="str">
-        <f t="shared" ref="K23:P23" si="9">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$23),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="L23" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>W</v>
       </c>
       <c r="M23" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>T</v>
       </c>
       <c r="N23" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>F</v>
       </c>
       <c r="O23" s="12" t="str">
-        <f t="shared" si="9"/>
         <v>S</v>
       </c>
       <c r="P23" s="12" t="str">
-        <f t="shared" si="9"/>
         <v>S</v>
       </c>
       <c r="Q23" s="11"/>
-      <c r="R23" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$23),"dddd"),1)</f>
+      <c r="R23" s="2" t="str" cm="1">
+        <f t="array" ref="R23:X23">week()</f>
         <v>M</v>
       </c>
       <c r="S23" s="2" t="str">
-        <f t="shared" ref="S23:X23" si="10">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$23),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="T23" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>W</v>
       </c>
       <c r="U23" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>T</v>
       </c>
       <c r="V23" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>F</v>
       </c>
       <c r="W23" s="12" t="str">
-        <f t="shared" si="10"/>
         <v>S</v>
       </c>
       <c r="X23" s="12" t="str">
-        <f t="shared" si="10"/>
         <v>S</v>
       </c>
       <c r="Y23" s="11"/>
-      <c r="Z23" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$23),"dddd"),1)</f>
+      <c r="Z23" s="2" t="str" cm="1">
+        <f t="array" ref="Z23:AF23">week()</f>
         <v>M</v>
       </c>
       <c r="AA23" s="2" t="str">
-        <f t="shared" ref="AA23:AF23" si="11">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$23),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="AB23" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>W</v>
       </c>
       <c r="AC23" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>T</v>
       </c>
       <c r="AD23" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>F</v>
       </c>
       <c r="AE23" s="12" t="str">
-        <f t="shared" si="11"/>
         <v>S</v>
       </c>
       <c r="AF23" s="12" t="str">
-        <f t="shared" si="11"/>
         <v>S</v>
       </c>
       <c r="AG23" s="9"/>
@@ -3605,7 +3533,7 @@
       </c>
       <c r="B2" s="13">
         <f ca="1">NOW()</f>
-        <v>46226.525753009257</v>
+        <v>46233.603531944442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>